<commit_message>
Update vendor #1/#2 UPC list (12 new part #s)
Owner's updated file: tab #1 adds 202-4-10=2XX/5XX/10XX,
31-1-3=2XX/5XX/10XX, 31-1-5=5XX/25XX, 43-4-11=1X/2X, 43-4-12=1X/2X.
Nothing removed or changed; no UPC points to two part #s. Both tabs are
read. 475 part #s now in data/upc and the Worker's scanner list.

keep-working: 1 check.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YD54BD5gJNAgEPeNDysnFF
</commit_message>
<xml_diff>
--- a/data/upc/vendor-1-2-box-bag-upc.xlsx
+++ b/data/upc/vendor-1-2-box-bag-upc.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2310" uniqueCount="1154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2346" uniqueCount="1190">
   <si>
     <t>Part Number</t>
   </si>
@@ -3474,6 +3474,114 @@
   </si>
   <si>
     <t>00810139937142</t>
+  </si>
+  <si>
+    <t>202-4-10=2XX</t>
+  </si>
+  <si>
+    <t>840428935962</t>
+  </si>
+  <si>
+    <t>840428935931</t>
+  </si>
+  <si>
+    <t>202-4-10=5XX</t>
+  </si>
+  <si>
+    <t>840428935979</t>
+  </si>
+  <si>
+    <t>840428935948</t>
+  </si>
+  <si>
+    <t>202-4-10=10XX</t>
+  </si>
+  <si>
+    <t>840428935986</t>
+  </si>
+  <si>
+    <t>840428935955</t>
+  </si>
+  <si>
+    <t>31-1-3=2XX</t>
+  </si>
+  <si>
+    <t>840428920142</t>
+  </si>
+  <si>
+    <t>840428920111</t>
+  </si>
+  <si>
+    <t>31-1-3=5XX</t>
+  </si>
+  <si>
+    <t>840428920159</t>
+  </si>
+  <si>
+    <t>840428920128</t>
+  </si>
+  <si>
+    <t>31-1-3=10XX</t>
+  </si>
+  <si>
+    <t>840428920166</t>
+  </si>
+  <si>
+    <t>840428920135</t>
+  </si>
+  <si>
+    <t>31-1-5=5XX</t>
+  </si>
+  <si>
+    <t>00840428940232</t>
+  </si>
+  <si>
+    <t>840428940218</t>
+  </si>
+  <si>
+    <t>31-1-5=25XX</t>
+  </si>
+  <si>
+    <t>00840428940249</t>
+  </si>
+  <si>
+    <t>840428940225</t>
+  </si>
+  <si>
+    <t>43-4-11=1X</t>
+  </si>
+  <si>
+    <t>840428944988</t>
+  </si>
+  <si>
+    <t>840428945008</t>
+  </si>
+  <si>
+    <t>43-4-11=2X</t>
+  </si>
+  <si>
+    <t>840428945022</t>
+  </si>
+  <si>
+    <t>840428945046</t>
+  </si>
+  <si>
+    <t>43-4-12=1X</t>
+  </si>
+  <si>
+    <t>840428944995</t>
+  </si>
+  <si>
+    <t>840428945015</t>
+  </si>
+  <si>
+    <t>43-4-12=2X</t>
+  </si>
+  <si>
+    <t>840428945039</t>
+  </si>
+  <si>
+    <t>840428945053</t>
   </si>
 </sst>
 </file>
@@ -3483,7 +3591,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="000000000000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -3507,6 +3615,11 @@
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12.0"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="6">
@@ -3541,7 +3654,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border/>
     <border>
       <left style="thin">
@@ -3568,11 +3681,23 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="40">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -3672,6 +3797,27 @@
     <xf borderId="0" fillId="2" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf quotePrefix="1" borderId="1" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf quotePrefix="1" borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="4" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -3731,7 +3877,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:C614" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:C626" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="3">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -9869,6 +10015,138 @@
         <v>1153</v>
       </c>
     </row>
+    <row r="615">
+      <c r="A615" s="33" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B615" s="33" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C615" s="34" t="s">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="33" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B616" s="33" t="s">
+        <v>1158</v>
+      </c>
+      <c r="C616" s="35" t="s">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="33" t="s">
+        <v>1160</v>
+      </c>
+      <c r="B617" s="33" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C617" s="34" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="36" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B618" s="36" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C618" s="37" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="38" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B619" s="38" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C619" s="39" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="36" t="s">
+        <v>1169</v>
+      </c>
+      <c r="B620" s="36" t="s">
+        <v>1170</v>
+      </c>
+      <c r="C620" s="37" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="36" t="s">
+        <v>1172</v>
+      </c>
+      <c r="B621" s="36" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C621" s="37" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="38" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B622" s="38" t="s">
+        <v>1176</v>
+      </c>
+      <c r="C622" s="39" t="s">
+        <v>1177</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="38" t="s">
+        <v>1178</v>
+      </c>
+      <c r="B623" s="38" t="s">
+        <v>1179</v>
+      </c>
+      <c r="C623" s="38" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="38" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B624" s="38" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C624" s="38" t="s">
+        <v>1183</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="38" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B625" s="38" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C625" s="38" t="s">
+        <v>1186</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="38" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B626" s="38" t="s">
+        <v>1188</v>
+      </c>
+      <c r="C626" s="38" t="s">
+        <v>1189</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>